<commit_message>
test: add Sprint 1 API test results and evidence
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-1-test-cases.xlsx
+++ b/docs/testing/sprint-1-test-cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01_Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\COIT20273\GradNavi\docs\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_16037A5C931E416AE01027FD425AB27C381DC958" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE2318F-837C-490B-88FC-4325EFDBFB2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11820" yWindow="21480" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -36,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1326" uniqueCount="642">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1402" uniqueCount="699">
   <si>
     <t>GradNavi Sprint 1 Test Dashboard</t>
   </si>
@@ -1962,6 +1960,177 @@
   </si>
   <si>
     <t>WBS 4.9 regression evidence</t>
+  </si>
+  <si>
+    <t>EV-048</t>
+  </si>
+  <si>
+    <t>201 Created; student account created successfully. Response returned id, email, first_name, last_name, and role, with no password fields exposed.</t>
+  </si>
+  <si>
+    <t>Valid student registration verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>400 Bad Request returned. Required-field validation correctly identified the missing last_name field and rejected the registration request.</t>
+  </si>
+  <si>
+    <t>EV-049</t>
+  </si>
+  <si>
+    <t>Missing required registration field validation verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>409 Conflict returned. Registration using an existing email was rejected with "A user with this email already exists." Duplicate account was not created.</t>
+  </si>
+  <si>
+    <t>Duplicate email registration validation verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-050</t>
+  </si>
+  <si>
+    <t>EV-051</t>
+  </si>
+  <si>
+    <t>201 Created; registration response returned only id, email, first_name, last_name, and role. Password, password_confirm, hashes, reset credentials, tokens, and other secrets were not exposed.</t>
+  </si>
+  <si>
+    <t>Registration response security verified via Postman on feature/sprint-3; sensitive authentication fields were not returned.</t>
+  </si>
+  <si>
+    <t>200 OK; valid credentials returned access token, refresh token, and authenticated user summary containing id, email, first_name, last_name, and role.</t>
+  </si>
+  <si>
+    <t>Valid student login verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-052</t>
+  </si>
+  <si>
+    <t>EV-053</t>
+  </si>
+  <si>
+    <t>401 Unauthorized; incorrect password returned a controlled invalid_credentials error and no access or refresh tokens were returned.</t>
+  </si>
+  <si>
+    <t>Invalid-password login handling verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>400 Bad Request; missing password returned the standard validation_error structure with password identified as a required field.</t>
+  </si>
+  <si>
+    <t>EV-054</t>
+  </si>
+  <si>
+    <t>Missing login credential validation verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>200 OK; authenticated request with a valid Bearer access token returned the current user's id, email, first_name, last_name, and role.</t>
+  </si>
+  <si>
+    <t>Current authenticated user retrieval verified via Postman on feature/sprint-3 using a valid access token.</t>
+  </si>
+  <si>
+    <t>EV-055</t>
+  </si>
+  <si>
+    <t>EV-056</t>
+  </si>
+  <si>
+    <t>401 Unauthorized; request without Authorization returned a not_authenticated error and no account data was returned.</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to the current-user endpoint was correctly rejected via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-057</t>
+  </si>
+  <si>
+    <t>200 OK; valid refresh token was accepted and a new access token was returned. A rotated refresh token was also issued.</t>
+  </si>
+  <si>
+    <t>Valid JWT refresh flow verified via Postman on feature/sprint-3; refresh-token rotation was observed.</t>
+  </si>
+  <si>
+    <t>EV-058</t>
+  </si>
+  <si>
+    <t>401 Unauthorized; invalid refresh token was rejected with token_not_valid error and no access token was issued.</t>
+  </si>
+  <si>
+    <t>Invalid JWT refresh token rejection verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-059</t>
+  </si>
+  <si>
+    <t>401 Unauthorized; previously invalidated refresh token was rejected with token_not_valid error and no access token was issued.</t>
+  </si>
+  <si>
+    <t>Reuse of the previously invalidated refresh token was rejected via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-060, EV-061</t>
+  </si>
+  <si>
+    <t>200 OK logout response received. Reusing the same refresh token returned 401 Unauthorized with token_not_valid, and no new access token was issued.</t>
+  </si>
+  <si>
+    <t>Logout and refresh-token blacklisting verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-062, EV-063</t>
+  </si>
+  <si>
+    <t>200 OK returned for both registered and unregistered email addresses with the same controlled password-reset message. No account existence information was disclosed.</t>
+  </si>
+  <si>
+    <t>Password reset request enumeration protection verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-064, EV-065</t>
+  </si>
+  <si>
+    <t>401 Unauthorized returned for invalid reset credentials with invalid_reset_token error. Subsequent login using the original password succeeded with 200 OK, confirming the password remained unchanged.</t>
+  </si>
+  <si>
+    <t>Invalid password-reset confirmation and unchanged-password behavior verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>401 Unauthorized; unauthenticated profile request returned a not_authenticated error and no profile data was returned.</t>
+  </si>
+  <si>
+    <t>EV-66</t>
+  </si>
+  <si>
+    <t>Unauthenticated access to the Student Profile endpoint was correctly rejected via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>EV-67,EV-68</t>
+  </si>
+  <si>
+    <t>400 Bad Request returned for an invalid profile field value. The API returned a validation_error stating that "INVALID_LEVEL" is not a valid proficiency_level choice. A subsequent GET returned 200 OK with skills remaining empty, confirming the invalid data was not persisted.</t>
+  </si>
+  <si>
+    <t>Invalid Student Profile field validation and non-persistence verified via Postman on feature/sprint-3.</t>
+  </si>
+  <si>
+    <t>200 OK; empty PATCH request was accepted and all Student Profile collections remained unchanged.</t>
+  </si>
+  <si>
+    <t>Empty Student Profile PATCH behavior verified via Postman on feature/sprint-3; no profile collections were modified.</t>
+  </si>
+  <si>
+    <t>EV-69</t>
+  </si>
+  <si>
+    <t>EV-70</t>
+  </si>
+  <si>
+    <t>400 Bad Request; attempted user_id ownership-field change was rejected with validation_error stating "This field is not allowed." The unsupported ownership field was not accepted.</t>
+  </si>
+  <si>
+    <t>Student Profile ownership-field protection verified via Postman on feature/sprint-3; client-supplied user_id was rejected as unsupported.</t>
   </si>
 </sst>
 </file>
@@ -1971,7 +2140,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -2014,6 +2183,18 @@
       <sz val="10"/>
       <color rgb="FF17365D"/>
       <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Aptos"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="9">
@@ -2102,7 +2283,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2170,6 +2351,16 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2180,7 +2371,197 @@
     <cellStyle name="Normal 6" xfId="5" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="Normal 7" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="37">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <name val="Aptos"/>
+        <scheme val="none"/>
+      </font>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F8FC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF3F8FC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -2289,13 +2670,6 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF3F8FC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <color rgb="FF8A5A00"/>
       </font>
@@ -2397,6 +2771,7 @@
           <a:lstStyle/>
           <a:p>
             <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>Sprint 1 Test Status</a:t>
             </a:r>
           </a:p>
@@ -2451,7 +2826,7 @@
                   <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>42</c:v>
+                  <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -2460,7 +2835,7 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>19</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2599,23 +2974,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Sprint1TestCases" displayName="Sprint1TestCases" ref="A1:O62" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Sprint1TestCases" displayName="Sprint1TestCases" ref="A1:O62" totalsRowShown="0" dataDxfId="0">
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Test ID"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Area"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Test Type"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Scenario"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Preconditions"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Test Steps"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Expected Result"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Actual Result"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Status"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Tester"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Test Date"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Evidence ID"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Defect Reference"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Notes"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Test ID" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Area" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Test Type" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Priority" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Scenario" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Preconditions" dataDxfId="10"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Test Steps" dataDxfId="9"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Expected Result" dataDxfId="8"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Actual Result" dataDxfId="7"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Status" dataDxfId="6"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Tester" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Test Date" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Evidence ID" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Defect Reference" dataDxfId="2"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Notes" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2935,7 +3310,7 @@
       </c>
       <c r="F4" s="5">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D4,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -2952,7 +3327,7 @@
       </c>
       <c r="B5" s="7">
         <f>COUNTIF('Test Cases'!J2:J62,"Pass")</f>
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1" t="s">
@@ -2964,7 +3339,7 @@
       </c>
       <c r="F5" s="5">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D5,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
@@ -2993,7 +3368,7 @@
       </c>
       <c r="F6" s="5">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D6,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
@@ -3022,7 +3397,7 @@
       </c>
       <c r="F7" s="5">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D7,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
@@ -3039,7 +3414,7 @@
       </c>
       <c r="B8" s="13">
         <f>COUNTIF('Test Cases'!J2:J62,"Not Run")</f>
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
@@ -3144,7 +3519,7 @@
       </c>
       <c r="B12" s="1" t="str">
         <f>IF(COUNTIFS('Test Cases'!D2:D62,"Critical",'Test Cases'!J2:J62,"Fail")+COUNTIFS('Test Cases'!D2:D62,"Critical",'Test Cases'!J2:J62,"Blocked")&gt;0,"NOT READY",IF(COUNTIFS('Test Cases'!D2:D62,"Critical",'Test Cases'!J2:J62,"Not Run")&gt;0,"PENDING","READY"))</f>
-        <v>PENDING</v>
+        <v>READY</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
@@ -3173,7 +3548,7 @@
       </c>
       <c r="B13" s="1" t="str">
         <f>IF(COUNTIFS('Test Cases'!C2:C62,"Integration",'Test Cases'!J2:J62,"Fail")+COUNTIFS('Test Cases'!C2:C62,"Integration",'Test Cases'!J2:J62,"Blocked")&gt;0,"NOT READY",IF(COUNTIFS('Test Cases'!C2:C62,"Integration",'Test Cases'!J2:J62,"Not Run")&gt;0,"PENDING","READY"))</f>
-        <v>PENDING</v>
+        <v>READY</v>
       </c>
       <c r="C13" s="1"/>
       <c r="D13" s="1" t="s">
@@ -3371,7 +3746,7 @@
       </c>
       <c r="J20" s="5">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H20,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>3</v>
+        <v>22</v>
       </c>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
@@ -3487,29 +3862,29 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <conditionalFormatting sqref="B12:B13">
-    <cfRule type="expression" dxfId="19" priority="1">
+    <cfRule type="expression" dxfId="36" priority="1">
       <formula>B12="READY"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="2">
+    <cfRule type="expression" dxfId="35" priority="2">
       <formula>B12="PENDING"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="3">
+    <cfRule type="expression" dxfId="34" priority="3">
       <formula>B12="NOT READY"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F4:F20">
-    <cfRule type="expression" dxfId="16" priority="4">
+    <cfRule type="expression" dxfId="33" priority="4">
       <formula>F4=E4</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="15" priority="5">
+    <cfRule type="expression" dxfId="32" priority="5">
       <formula>F4&lt;E4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J20:J23">
-    <cfRule type="expression" dxfId="14" priority="6">
+    <cfRule type="expression" dxfId="31" priority="6">
       <formula>J20=I20</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="7">
+    <cfRule type="expression" dxfId="30" priority="7">
       <formula>J20&lt;I20</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3615,15 +3990,25 @@
       <c r="H2" s="16" t="s">
         <v>417</v>
       </c>
-      <c r="I2" s="16"/>
+      <c r="I2" s="25" t="s">
+        <v>643</v>
+      </c>
       <c r="J2" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="23">
+        <v>46282</v>
+      </c>
+      <c r="M2" s="17" t="s">
+        <v>642</v>
+      </c>
       <c r="N2" s="16"/>
-      <c r="O2" s="16"/>
+      <c r="O2" s="25" t="s">
+        <v>644</v>
+      </c>
       <c r="P2" s="17" t="s">
         <v>34</v>
       </c>
@@ -3653,15 +4038,25 @@
       <c r="H3" s="16" t="s">
         <v>418</v>
       </c>
-      <c r="I3" s="16"/>
+      <c r="I3" s="25" t="s">
+        <v>645</v>
+      </c>
       <c r="J3" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K3" s="17"/>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L3" s="23">
+        <v>46282</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>646</v>
+      </c>
       <c r="N3" s="16"/>
-      <c r="O3" s="16"/>
+      <c r="O3" s="25" t="s">
+        <v>647</v>
+      </c>
       <c r="P3" s="17" t="s">
         <v>34</v>
       </c>
@@ -3691,15 +4086,25 @@
       <c r="H4" s="16" t="s">
         <v>419</v>
       </c>
-      <c r="I4" s="16"/>
+      <c r="I4" s="24" t="s">
+        <v>648</v>
+      </c>
       <c r="J4" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K4" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L4" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M4" s="17" t="s">
+        <v>650</v>
+      </c>
       <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
+      <c r="O4" s="24" t="s">
+        <v>649</v>
+      </c>
       <c r="P4" s="17" t="s">
         <v>34</v>
       </c>
@@ -3729,15 +4134,25 @@
       <c r="H5" s="16" t="s">
         <v>420</v>
       </c>
-      <c r="I5" s="16"/>
+      <c r="I5" s="25" t="s">
+        <v>652</v>
+      </c>
       <c r="J5" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L5" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M5" s="17" t="s">
+        <v>651</v>
+      </c>
       <c r="N5" s="16"/>
-      <c r="O5" s="16"/>
+      <c r="O5" s="25" t="s">
+        <v>653</v>
+      </c>
       <c r="P5" s="17" t="s">
         <v>34</v>
       </c>
@@ -3767,15 +4182,25 @@
       <c r="H6" s="16" t="s">
         <v>421</v>
       </c>
-      <c r="I6" s="16"/>
+      <c r="I6" s="24" t="s">
+        <v>654</v>
+      </c>
       <c r="J6" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K6" s="17"/>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L6" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>656</v>
+      </c>
       <c r="N6" s="16"/>
-      <c r="O6" s="16"/>
+      <c r="O6" s="24" t="s">
+        <v>655</v>
+      </c>
       <c r="P6" s="17" t="s">
         <v>34</v>
       </c>
@@ -3805,15 +4230,25 @@
       <c r="H7" s="16" t="s">
         <v>422</v>
       </c>
-      <c r="I7" s="16"/>
+      <c r="I7" s="25" t="s">
+        <v>658</v>
+      </c>
       <c r="J7" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L7" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>657</v>
+      </c>
       <c r="N7" s="16"/>
-      <c r="O7" s="16"/>
+      <c r="O7" s="25" t="s">
+        <v>659</v>
+      </c>
       <c r="P7" s="17" t="s">
         <v>34</v>
       </c>
@@ -3843,15 +4278,25 @@
       <c r="H8" s="16" t="s">
         <v>423</v>
       </c>
-      <c r="I8" s="16"/>
+      <c r="I8" s="24" t="s">
+        <v>660</v>
+      </c>
       <c r="J8" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L8" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M8" s="17" t="s">
+        <v>661</v>
+      </c>
       <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
+      <c r="O8" s="25" t="s">
+        <v>662</v>
+      </c>
       <c r="P8" s="17" t="s">
         <v>34</v>
       </c>
@@ -3881,15 +4326,25 @@
       <c r="H9" s="16" t="s">
         <v>424</v>
       </c>
-      <c r="I9" s="16"/>
+      <c r="I9" s="25" t="s">
+        <v>663</v>
+      </c>
       <c r="J9" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L9" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M9" s="17" t="s">
+        <v>665</v>
+      </c>
       <c r="N9" s="16"/>
-      <c r="O9" s="16"/>
+      <c r="O9" s="25" t="s">
+        <v>664</v>
+      </c>
       <c r="P9" s="17" t="s">
         <v>34</v>
       </c>
@@ -3919,15 +4374,25 @@
       <c r="H10" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="I10" s="16"/>
+      <c r="I10" s="25" t="s">
+        <v>667</v>
+      </c>
       <c r="J10" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L10" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M10" s="17" t="s">
+        <v>666</v>
+      </c>
       <c r="N10" s="16"/>
-      <c r="O10" s="16"/>
+      <c r="O10" s="25" t="s">
+        <v>668</v>
+      </c>
       <c r="P10" s="17" t="s">
         <v>34</v>
       </c>
@@ -3957,15 +4422,25 @@
       <c r="H11" s="16" t="s">
         <v>425</v>
       </c>
-      <c r="I11" s="16"/>
+      <c r="I11" s="25" t="s">
+        <v>670</v>
+      </c>
       <c r="J11" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L11" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M11" s="17" t="s">
+        <v>669</v>
+      </c>
       <c r="N11" s="16"/>
-      <c r="O11" s="16"/>
+      <c r="O11" s="25" t="s">
+        <v>671</v>
+      </c>
       <c r="P11" s="17" t="s">
         <v>34</v>
       </c>
@@ -3995,15 +4470,25 @@
       <c r="H12" s="16" t="s">
         <v>426</v>
       </c>
-      <c r="I12" s="16"/>
+      <c r="I12" s="25" t="s">
+        <v>673</v>
+      </c>
       <c r="J12" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L12" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>672</v>
+      </c>
       <c r="N12" s="16"/>
-      <c r="O12" s="16"/>
+      <c r="O12" s="25" t="s">
+        <v>674</v>
+      </c>
       <c r="P12" s="17" t="s">
         <v>34</v>
       </c>
@@ -4033,15 +4518,25 @@
       <c r="H13" s="16" t="s">
         <v>427</v>
       </c>
-      <c r="I13" s="16"/>
+      <c r="I13" s="25" t="s">
+        <v>676</v>
+      </c>
       <c r="J13" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L13" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M13" s="17" t="s">
+        <v>675</v>
+      </c>
       <c r="N13" s="16"/>
-      <c r="O13" s="16"/>
+      <c r="O13" s="25" t="s">
+        <v>677</v>
+      </c>
       <c r="P13" s="17" t="s">
         <v>34</v>
       </c>
@@ -4071,15 +4566,25 @@
       <c r="H14" s="16" t="s">
         <v>428</v>
       </c>
-      <c r="I14" s="16"/>
+      <c r="I14" s="25" t="s">
+        <v>679</v>
+      </c>
       <c r="J14" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K14" s="17"/>
-      <c r="L14" s="17"/>
-      <c r="M14" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14" s="23">
+        <v>46283</v>
+      </c>
+      <c r="M14" s="17" t="s">
+        <v>678</v>
+      </c>
       <c r="N14" s="16"/>
-      <c r="O14" s="16"/>
+      <c r="O14" s="25" t="s">
+        <v>680</v>
+      </c>
       <c r="P14" s="17" t="s">
         <v>34</v>
       </c>
@@ -4109,15 +4614,25 @@
       <c r="H15" s="16" t="s">
         <v>429</v>
       </c>
-      <c r="I15" s="16"/>
+      <c r="I15" s="25" t="s">
+        <v>682</v>
+      </c>
       <c r="J15" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K15" s="17"/>
-      <c r="L15" s="17"/>
-      <c r="M15" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15" s="23">
+        <v>46286</v>
+      </c>
+      <c r="M15" s="17" t="s">
+        <v>681</v>
+      </c>
       <c r="N15" s="16"/>
-      <c r="O15" s="16"/>
+      <c r="O15" s="25" t="s">
+        <v>683</v>
+      </c>
       <c r="P15" s="17" t="s">
         <v>34</v>
       </c>
@@ -4147,15 +4662,25 @@
       <c r="H16" s="16" t="s">
         <v>430</v>
       </c>
-      <c r="I16" s="16"/>
+      <c r="I16" s="25" t="s">
+        <v>685</v>
+      </c>
       <c r="J16" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K16" s="17"/>
-      <c r="L16" s="17"/>
-      <c r="M16" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16" s="23">
+        <v>46286</v>
+      </c>
+      <c r="M16" s="17" t="s">
+        <v>684</v>
+      </c>
       <c r="N16" s="16"/>
-      <c r="O16" s="16"/>
+      <c r="O16" s="25" t="s">
+        <v>686</v>
+      </c>
       <c r="P16" s="17" t="s">
         <v>34</v>
       </c>
@@ -4233,15 +4758,25 @@
       <c r="H18" s="16" t="s">
         <v>126</v>
       </c>
-      <c r="I18" s="16"/>
+      <c r="I18" s="26" t="s">
+        <v>687</v>
+      </c>
       <c r="J18" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K18" s="17"/>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K18" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18" s="23">
+        <v>46286</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>688</v>
+      </c>
       <c r="N18" s="16"/>
-      <c r="O18" s="16"/>
+      <c r="O18" s="25" t="s">
+        <v>689</v>
+      </c>
       <c r="P18" s="17" t="s">
         <v>34</v>
       </c>
@@ -4367,15 +4902,25 @@
       <c r="H21" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="I21" s="16"/>
+      <c r="I21" s="26" t="s">
+        <v>691</v>
+      </c>
       <c r="J21" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K21" s="17"/>
-      <c r="L21" s="17"/>
-      <c r="M21" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L21" s="23">
+        <v>46286</v>
+      </c>
+      <c r="M21" s="17" t="s">
+        <v>690</v>
+      </c>
       <c r="N21" s="16"/>
-      <c r="O21" s="16"/>
+      <c r="O21" s="25" t="s">
+        <v>692</v>
+      </c>
       <c r="P21" s="17" t="s">
         <v>34</v>
       </c>
@@ -4405,15 +4950,25 @@
       <c r="H22" s="16" t="s">
         <v>436</v>
       </c>
-      <c r="I22" s="16"/>
+      <c r="I22" s="25" t="s">
+        <v>693</v>
+      </c>
       <c r="J22" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K22" s="17"/>
-      <c r="L22" s="17"/>
-      <c r="M22" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K22" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22" s="23">
+        <v>46286</v>
+      </c>
+      <c r="M22" s="17" t="s">
+        <v>695</v>
+      </c>
       <c r="N22" s="16"/>
-      <c r="O22" s="16"/>
+      <c r="O22" s="25" t="s">
+        <v>694</v>
+      </c>
       <c r="P22" s="17" t="s">
         <v>34</v>
       </c>
@@ -4443,15 +4998,25 @@
       <c r="H23" s="16" t="s">
         <v>437</v>
       </c>
-      <c r="I23" s="16"/>
+      <c r="I23" s="25" t="s">
+        <v>697</v>
+      </c>
       <c r="J23" s="17" t="s">
-        <v>14</v>
-      </c>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
+        <v>8</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L23" s="23">
+        <v>46286</v>
+      </c>
+      <c r="M23" s="17" t="s">
+        <v>696</v>
+      </c>
       <c r="N23" s="16"/>
-      <c r="O23" s="16"/>
+      <c r="O23" s="16" t="s">
+        <v>698</v>
+      </c>
       <c r="P23" s="17" t="s">
         <v>34</v>
       </c>
@@ -6327,37 +6892,43 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:P62">
-    <cfRule type="expression" dxfId="12" priority="7">
+  <phoneticPr fontId="10" type="noConversion"/>
+  <conditionalFormatting sqref="A17:P17 N16 J2:N15 A2:H16 J16:L16 P2:P16 A18:H18 J18:N18 P18 A19:P20 J21:N22 P21:P22 A24:P62 A21:H23 J23:P23">
+    <cfRule type="expression" dxfId="17" priority="8">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D62">
-    <cfRule type="expression" dxfId="11" priority="8">
+    <cfRule type="expression" dxfId="29" priority="9">
       <formula>D2="Critical"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="10" priority="9">
+    <cfRule type="expression" dxfId="28" priority="10">
       <formula>D2="High"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="9" priority="10">
+    <cfRule type="expression" dxfId="27" priority="11">
       <formula>D2="Medium"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="8" priority="11">
+    <cfRule type="expression" dxfId="26" priority="12">
       <formula>D2="Low"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J62">
-    <cfRule type="expression" dxfId="7" priority="12">
+    <cfRule type="expression" dxfId="25" priority="13">
       <formula>J2="Pass"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="6" priority="13">
+    <cfRule type="expression" dxfId="24" priority="14">
       <formula>J2="Fail"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="14">
+    <cfRule type="expression" dxfId="23" priority="15">
       <formula>J2="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="15">
+    <cfRule type="expression" dxfId="22" priority="16">
       <formula>J2="Not Run"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M16">
+    <cfRule type="expression" dxfId="16" priority="1">
+      <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -6372,8 +6943,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -9162,7 +9734,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:H48">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="21" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9607,17 +10179,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:D18">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:G18">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="19" priority="2">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2:J18">
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="18" priority="3">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>